<commit_message>
LIVE del martes 27 por Zoom privado: plan Fase 1 y plan de correos
- Nombre exacto: "LIVE GRATIS · Hipnosis para HACKEAR bloqueos con el DINERO".
- Registro: formulario de Brevo -> comunidad de WhatsApp -> link de Zoom por correo y WhatsApp.
- CTA de invitación: "Regístrate gratis: link en mi perfil y te mando el acceso por correo y WhatsApp".
- Estructura del LIVE adaptada a Zoom (chat, cámara, audífonos, micrófono).
- Correos E4 y E5 con el marcador [LINK DE ZOOM]; E4/E5 solo a registrados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XHpWW3cNoPrwBL8CwPdgsU
</commit_message>
<xml_diff>
--- a/nica-apify/briefs/plan-correos-2026-10-24.xlsx
+++ b/nica-apify/briefs/plan-correos-2026-10-24.xlsx
@@ -539,7 +539,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Activaciones Robóticas Millonarias · $500 MXN (Hotmart) y, solo el martes 27, Pack de Autohipnosis BNQ™ (5 audios) a $2,500 hasta las 21:00; después $3,000.</t>
+          <t>Activaciones Robóticas Millonarias · $500 MXN (Hotmart) y, solo el martes 27, Pack de Hipnosis BNQ™ (5 audios) a $2,500 solo durante el LIVE (cierra a las 21:00); después $3,000. En el LIVE se ofrece primero Robóticas y la venta principal es el Pack.</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Martes 27 oct · 10:00 AM y 7:00 PM CDMX · TikTok · 'Activación en tiempo real · Hipnosis para eliminar bloqueos con el dinero'. Registro: grupo de WhatsApp (botón 1 de Linktree).</t>
+          <t>Martes 27 oct · 10:00 AM y 7:00 PM CDMX · ZOOM privado (solo para registrados) · 'LIVE GRATIS · Hipnosis para HACKEAR bloqueos con el DINERO'. Registro: formulario de Brevo (nombre, correo, país; botón 1 de Linktree y banner en www.mabradiante.com) → comunidad de WhatsApp → link de Zoom por correo (E4 y E5) y por WhatsApp.</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>TODOS · NO ABRIERON E1 · ABRIERON (abrió o hizo clic en cualquier correo de esta serie) · RESPONDIERON SÍ (los marcas a mano) · REGISTRADOS (leads del formulario de anuncios, se suben a Brevo cada día) · INACTIVOS (desde el 9 nov, ya no se les escribe).</t>
+          <t>TODOS · NO ABRIERON E1 · ABRIERON (abrió o hizo clic en cualquier correo de esta serie) · RESPONDIERON SÍ (los marcas a mano) · REGISTRADOS (formulario de Brevo del LIVE + leads del formulario de anuncios, que se suben a Brevo cada día) · INACTIVOS (desde el 9 nov, ya no se les escribe).</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Meta: 2% o más de los enviados. E3–E5: clics a Linktree; E8–E9: clics a Hotmart.</t>
+          <t>Meta: 2% o más de los enviados. E3: clics a Linktree (registro); E4–E5: clics al link de Zoom; E8–E9: clics a Hotmart.</t>
         </is>
       </c>
     </row>
@@ -699,7 +699,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Clics de E3–E5 en Linktree (botón 1). Comparar con el total de clics de Linktree de la semana.</t>
+          <t>Contactos nuevos del formulario de Brevo del LIVE + clics de E3 en Linktree (botón 1). Comparar con el total de clics de Linktree de la semana.</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Que entren al grupo de WhatsApp del LIVE (registro). Valor primero: hackeo para hacer hoy.</t>
+          <t>Que se registren al LIVE por Zoom (formulario de Brevo, botón 1 de Linktree) y entren a la comunidad de WhatsApp. Valor primero: hackeo para hacer hoy.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Listo · falta [TU HISTORIA] y que el grupo ya sea el botón 1</t>
+          <t>Listo · falta [TU HISTORIA] y que el formulario de registro ya sea el botón 1</t>
         </is>
       </c>
     </row>
@@ -953,7 +953,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>ABRIERON (E1, E2 o E3) + REGISTRADOS</t>
+          <t>REGISTRADOS (formulario del LIVE + anuncios)</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Recordatorio del día y cómo prepararse. Más asistencia a las 10 AM.</t>
+          <t>Recordatorio del día, cómo prepararse y el link de Zoom. Más asistencia a las 10 AM.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -978,7 +978,7 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Listo para pegar</t>
+          <t>Falta pegar el [LINK DE ZOOM]</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>REGISTRADOS + ABRIERON E4</t>
+          <t>REGISTRADOS (formulario del LIVE + anuncios)</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Llevar gente al segundo LIVE (7 PM), donde se cierra la venta.</t>
+          <t>Llevar gente al segundo LIVE (7 PM, por Zoom), donde se cierra la venta. Lleva el link de Zoom.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Listo para pegar</t>
+          <t>Falta pegar el [LINK DE ZOOM]</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
 Si es un sí, contesta este correo con una sola palabra: SÍ.
 Así sé que estás del otro lado (y tu correo deja de mandarme a promociones).
 Si ya no te interesa, no pasa nada: abajo está el enlace para darte de baja, sin culpa.
-Un adelanto para quien se quede: el martes 27 de octubre hago una activación en tiempo real, gratis, en TikTok. Te doy los detalles el lunes.
+Un adelanto para quien se quede: el martes 27 de octubre hago un LIVE gratis y privado por Zoom: Hipnosis para hackear bloqueos con el dinero. Te doy los detalles el lunes.
 Con cariño,
 Mabel Soriano
 @mabradiante · Método BNQ™</t>
@@ -1591,7 +1591,7 @@
 Te lo pregunto corto: ¿quieres seguir recibiendo mis hackeos de biohacking y neurorreprogramación?
 Contesta con una palabra: SÍ.
 Si no, abajo está el enlace para darte de baja. Prefiero escribirle a quien sí quiere estar aquí.
-PD: el martes 27 hago una activación en vivo, gratis, para los bloqueos con el dinero. Si contestas SÍ, te mando los detalles.
+PD: el martes 27 hago un LIVE gratis y privado por Zoom para hackear los bloqueos con el dinero. Si contestas SÍ, te mando los detalles.
 Con cariño,
 Mabel Soriano
 @mabradiante · Método BNQ™</t>
@@ -1641,7 +1641,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Martes 27 · 10 AM y 7 PM (CDMX) · en vivo en TikTok, sin costo</t>
+          <t>Martes 27 · 10 AM y 7 PM (CDMX) · en vivo por Zoom, privado y sin costo</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -1651,8 +1651,8 @@
 No es flojera ni mala suerte. Muchas veces es un programa: tu cuerpo aprendió a vivir el dinero en modo alarma, y tu mente repite lo que escuchó en casa.
 [TU HISTORIA con el dinero, en 2 o 3 líneas]
 Por eso mañana hago algo especial en vivo:
-ACTIVACIÓN EN TIEMPO REAL · Hipnosis para eliminar bloqueos con el dinero
-Martes 27 de octubre, en mi TikTok
+LIVE GRATIS · Hipnosis para HACKEAR bloqueos con el DINERO
+Martes 27 de octubre, por Zoom (privado: solo para quien se registra)
 10:00 AM o 7:00 PM (hora CDMX): elige una
 Colombia 11 AM / 8 PM · Argentina 1 PM / 10 PM · España 5 PM
 Lo trabajamos con el Método BNQ™:
@@ -1662,7 +1662,7 @@
 Tu hackeo para hoy (30 segundos):
 Mano en el pecho. Inhala en 4, sostén en 4, suelta en 6. Y di 3 veces: "Hoy me permito recibir con calma."
 Nota qué sientes en el cuerpo al decirlo. Eso es justo lo que trabajamos mañana.
-Para no perdértelo, entra al grupo de WhatsApp del LIVE (es el primer botón de mi Linktree). Ahí aviso cuando empezamos.
+Para entrar, regístrate gratis con tu nombre, tu correo y tu país (es el primer botón de mi Linktree y también está en www.mabradiante.com). Al registrarte entras a mi comunidad de WhatsApp y te mando el link de Zoom por correo y por WhatsApp.
 Es una práctica de bienestar: no sustituye atención médica ni psicológica.
 Con cariño,
 Mabel Soriano
@@ -1671,17 +1671,17 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Quiero entrar al grupo del LIVE</t>
+          <t>Quiero registrarme gratis al LIVE</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>https://linktr.ee/mabradiante  (botón 1 = grupo de WhatsApp del LIVE)</t>
+          <t>https://linktr.ee/mabradiante  (botón 1 = formulario de registro de Brevo)</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Listo · falta [TU HISTORIA] y que el grupo ya sea el botón 1</t>
+          <t>Listo · falta [TU HISTORIA] y que el formulario de registro ya sea el botón 1</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1698,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>ABRIERON (E1, E2 o E3) + REGISTRADOS</t>
+          <t>REGISTRADOS (formulario del LIVE + anuncios)</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1713,20 +1713,23 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Ten audífonos y un lugar tranquilo. Dura 1 hora.</t>
+          <t>Aquí va tu link de Zoom. Ten audífonos y un lugar tranquilo. Dura 1 hora.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Hola, {{ contact.FIRSTNAME | default : "" }}:
-Hoy es la activación en vivo: Hipnosis para eliminar bloqueos con el dinero.
-10:00 AM y 7:00 PM (hora CDMX), en mi TikTok. Elige la que te acomode.
+Hoy es el LIVE GRATIS · Hipnosis para HACKEAR bloqueos con el DINERO.
+10:00 AM y 7:00 PM (hora CDMX), por Zoom. Elige la que te acomode.
+Tu link de Zoom (es privado: no lo compartas en redes):
+[LINK DE ZOOM]
 Para que la vivas completa:
 1. Audífonos y un lugar donde nadie te interrumpa.
 2. Nunca manejando ni haciendo otra cosa.
 3. Un vaso de agua y una hoja para escribir lo que sientas.
+4. Entra 5 minutos antes, con el micrófono en silencio. La cámara es opcional.
 Quédate hasta el final: al cerrar hacemos un decreto juntas y juntos.
-Si aún no estás en el grupo de WhatsApp, entra aquí (primer botón). Ahí aviso en cuanto empiece.
+Si aún no estás en la comunidad de WhatsApp, entra desde el primer botón de mi Linktree: ahí también te mando el link de Zoom y aviso en cuanto abra la sala.
 Es una práctica de bienestar: no sustituye atención médica ni psicológica.
 Con cariño,
 Mabel Soriano
@@ -1735,17 +1738,17 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Entrar al grupo y que me avisen</t>
+          <t>Entrar al LIVE por Zoom</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>https://linktr.ee/mabradiante</t>
+          <t>[LINK DE ZOOM]</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Listo para pegar</t>
+          <t>Falta pegar el [LINK DE ZOOM]</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1765,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>REGISTRADOS + ABRIERON E4</t>
+          <t>REGISTRADOS (formulario del LIVE + anuncios)</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1783,11 +1786,13 @@
       <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Hola, {{ contact.FIRSTNAME | default : "" }}:
-En 1 hora empezamos la segunda activación en vivo: 7:00 PM, hora CDMX, en mi TikTok.
+En 1 hora empezamos el segundo LIVE: 7:00 PM, hora CDMX, por Zoom.
+Tu link de Zoom (privado, solo para ti):
+[LINK DE ZOOM]
 Si en la mañana no pudiste, esta es tu oportunidad. Y si ya estuviste, repetirla le ayuda a tu cerebro a fijar el nuevo programa.
-Busca un lugar tranquilo, ponte audífonos y entra 5 minutos antes.
+Busca un lugar tranquilo, ponte audífonos y entra 5 minutos antes, con el micrófono en silencio.
 Al final te cuento cómo seguir practicando en casa.
-El aviso de "estoy en vivo" lo mando al grupo de WhatsApp (primer botón):
+El aviso de "ya abrimos la sala" también lo mando a la comunidad de WhatsApp.
 Con cariño,
 Mabel Soriano
 @mabradiante · Método BNQ™</t>
@@ -1795,17 +1800,17 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Entrar al grupo del LIVE</t>
+          <t>Entrar al LIVE de las 7 PM por Zoom</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>https://linktr.ee/mabradiante</t>
+          <t>[LINK DE ZOOM]</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Listo para pegar</t>
+          <t>Falta pegar el [LINK DE ZOOM]</t>
         </is>
       </c>
     </row>
@@ -1843,7 +1848,7 @@
       <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Hola, {{ contact.FIRSTNAME | default : "" }}:
-Gracias por estar hoy (o por querer estar). Leí cada palabra que escribieron en el LIVE.
+Gracias por estar hoy (o por querer estar). Leí cada palabra que escribieron en el chat de Zoom.
 Lo que hicimos hoy fue un primer cambio de estado. Para que el programa nuevo se quede, se practica. Por eso armé el Pack de Autohipnosis BNQ™: 5 audios, cada uno con el proceso BIO-Hardware → NEURO-Software → QUANTUM-Activación:
 1. Dinero: Hipnosis para hackear bloqueos con el dinero.
 2. Relaciones: Hipnosis para hackear relaciones tóxicas.
@@ -1909,7 +1914,7 @@
       <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Hola, {{ contact.FIRSTNAME | default : "" }}:
-Ayer, en las dos activaciones, pasó algo bonito. Algunas cosas que escribieron:
+Ayer, en las dos activaciones, pasó algo bonito. Algunas cosas que escribieron en el chat de Zoom:
 [PEGA 2 o 3 COMENTARIOS REALES DEL LIVE, solo con permiso o sin nombre]
 Lo que sientes después de una hipnosis se puede ir en 2 días si no lo practicas. Tu cerebro vuelve al programa viejo porque es el camino conocido.
 Hackeo para mantenerlo (1 minuto, en la mañana):
@@ -2221,7 +2226,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>[FECHA Y HORA DEL LIVE · por confirmar] · en vivo en TikTok, sin costo</t>
+          <t>[FECHA Y HORA DEL LIVE · por confirmar] · en vivo, sin costo ([PLATAFORMA · por confirmar])</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -2231,9 +2236,9 @@
 Por eso te invito a mi próxima activación en vivo:
 HACKEA Y ACTIVA TU MENTE SUBCONSCIENTE Y TUS HABILIDADES DORMIDAS
 Activación en tiempo real, sin costo
-[FECHA Y HORA · por confirmar] (hora CDMX), en mi TikTok
+[FECHA Y HORA · por confirmar] (hora CDMX), [PLATAFORMA · por confirmar: ¿Zoom privado como el del 27?]
 [TU HISTORIA: una habilidad que despertaste tú]
-Entra al grupo de WhatsApp (primer botón de mi Linktree) para que te avise cuando empiece.
+Regístrate gratis en el primer botón de mi Linktree y te mando el acceso por correo y WhatsApp.
 Es una práctica de bienestar: no sustituye atención médica ni psicológica.
 Con cariño,
 Mabel Soriano
@@ -2242,7 +2247,7 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Entrar al grupo del LIVE</t>
+          <t>Quiero registrarme gratis al LIVE</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -2707,7 +2712,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Para el LIVE, el aviso fuerte va en el grupo de WhatsApp y en TikTok; el correo queda de apoyo.</t>
+          <t>Para el LIVE, el aviso fuerte va en la comunidad de WhatsApp (con el link de Zoom); el correo queda de apoyo. En redes solo se invita a registrarse.</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -2815,7 +2820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3011,7 +3016,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Fase 2: fecha, hora y fórmula(s) del LIVE de atracción.</t>
+          <t>Fase 2: fecha, hora, fórmula(s) y plataforma del LIVE de atracción (¿Zoom privado como el del 27?).</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -3082,6 +3087,26 @@
       <c r="D15" s="3" t="inlineStr">
         <is>
           <t>Sin números no hay siguiente plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Crear las 2 reuniones de Zoom (10 AM y 7 PM) y pegar el link donde dice [LINK DE ZOOM] en E4 y E5 (y mandarlo a la comunidad de WhatsApp).</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Antes del lun 26</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Sin link de Zoom, E4 y E5 no se envían.</t>
         </is>
       </c>
     </row>

</xml_diff>